<commit_message>
chore: modify(plc service, operate log)
</commit_message>
<xml_diff>
--- a/Document/RLC_IO_Protocol_Map.xlsx
+++ b/Document/RLC_IO_Protocol_Map.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\1. RLC\RLC_LoadBank_SeparateVer\Document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E0E87811-7313-4E2C-B1BB-8F6922471FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A30C358-4D05-4BC1-A14B-9B3FBF8AC2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_분석요약" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="07_인터락_시퀀스" sheetId="8" r:id="rId8"/>
     <sheet name="08_미결정사항" sheetId="9" r:id="rId9"/>
     <sheet name="09_모듈요약" sheetId="10" r:id="rId10"/>
+    <sheet name="10_장비 리스트업" sheetId="11" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_분석요약'!$A$1:$B$10</definedName>
@@ -37,12 +38,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09_모듈요약'!$A$1:$F$20</definedName>
   </definedNames>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6509" uniqueCount="1059">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6548" uniqueCount="1098">
   <si>
     <t>항목</t>
   </si>
@@ -3219,12 +3219,144 @@
   </si>
   <si>
     <t>Channels</t>
+  </si>
+  <si>
+    <t>Device</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>ISEM2-WHRUH_01</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>ISEM2-WHRUH_02</t>
+  </si>
+  <si>
+    <t>ISEM2-WHRUH_03</t>
+  </si>
+  <si>
+    <t>ISEM2-WHRUH_04</t>
+  </si>
+  <si>
+    <t>ISEM2-WHRUH_05</t>
+  </si>
+  <si>
+    <t>ISEM2-WHRUH_06</t>
+  </si>
+  <si>
+    <t>ISEM2-WHRUH_07</t>
+  </si>
+  <si>
+    <t>ISEM2-WHRUH_08</t>
+  </si>
+  <si>
+    <t>ISEM2-WHRUH_09</t>
+  </si>
+  <si>
+    <t>ISEM2-WHRUH_10</t>
+  </si>
+  <si>
+    <t>GIMAC1000_01</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>GIMAC1000_02</t>
+  </si>
+  <si>
+    <t>GIMAC1000_03</t>
+  </si>
+  <si>
+    <t>GIMAC1000_04</t>
+  </si>
+  <si>
+    <t>IP</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>PORT</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>SERIAL NUMBER</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>251217-2613.0004</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>192.168.1.11</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>192.168.1.10</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>192.168.1.12</t>
+  </si>
+  <si>
+    <t>192.168.1.13</t>
+  </si>
+  <si>
+    <t>192.168.1.14</t>
+  </si>
+  <si>
+    <t>192.168.1.15</t>
+  </si>
+  <si>
+    <t>192.168.1.16</t>
+  </si>
+  <si>
+    <t>192.168.1.17</t>
+  </si>
+  <si>
+    <t>192.168.1.18</t>
+  </si>
+  <si>
+    <t>192.168.1.19</t>
+  </si>
+  <si>
+    <t>192.168.1.20</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>192.168.1.21</t>
+  </si>
+  <si>
+    <t>192.168.1.22</t>
+  </si>
+  <si>
+    <t>192.168.1.23</t>
+  </si>
+  <si>
+    <t>PLC_01</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>PLC_02</t>
+  </si>
+  <si>
+    <t>PLC_03</t>
+  </si>
+  <si>
+    <t>192.168.1.1</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>192.168.1.2</t>
+  </si>
+  <si>
+    <t>192.168.1.3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="178" formatCode="0_);[Red]\(0\)"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -3256,7 +3388,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3266,6 +3398,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -3296,12 +3446,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4119,6 +4290,298 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6C48EAB-8832-4C21-85B7-2FA35ACA6F68}">
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.875" customWidth="1"/>
+    <col min="2" max="2" width="10.5" customWidth="1"/>
+    <col min="4" max="4" width="16.75" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="27" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1074</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1075</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1076</v>
+      </c>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>1092</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>1095</v>
+      </c>
+      <c r="C2" s="5">
+        <v>502</v>
+      </c>
+      <c r="D2" s="5"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+    </row>
+    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>1093</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>1096</v>
+      </c>
+      <c r="C3" s="5">
+        <v>502</v>
+      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+    </row>
+    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>1094</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C4" s="5">
+        <v>502</v>
+      </c>
+      <c r="D4" s="5"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+    </row>
+    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>1079</v>
+      </c>
+      <c r="C5" s="3">
+        <v>502</v>
+      </c>
+      <c r="D5" s="4">
+        <v>6202012552304000</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>1078</v>
+      </c>
+      <c r="C6" s="3">
+        <v>502</v>
+      </c>
+      <c r="D6" s="4">
+        <v>6202012552304020</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>1080</v>
+      </c>
+      <c r="C7" s="3">
+        <v>502</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>1063</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>1081</v>
+      </c>
+      <c r="C8" s="3">
+        <v>502</v>
+      </c>
+      <c r="D8" s="4"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>1064</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C9" s="3">
+        <v>502</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>1083</v>
+      </c>
+      <c r="C10" s="3">
+        <v>502</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>1066</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>1084</v>
+      </c>
+      <c r="C11" s="3">
+        <v>502</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>1085</v>
+      </c>
+      <c r="C12" s="3">
+        <v>502</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+    </row>
+    <row r="13" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>1068</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C13" s="3">
+        <v>502</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>1069</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>1087</v>
+      </c>
+      <c r="C14" s="3">
+        <v>502</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+    </row>
+    <row r="15" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>1070</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>1088</v>
+      </c>
+      <c r="C15" s="7">
+        <v>502</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>1077</v>
+      </c>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C16" s="7">
+        <v>502</v>
+      </c>
+      <c r="D16" s="8"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="7" t="s">
+        <v>1072</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C17" s="7">
+        <v>502</v>
+      </c>
+      <c r="D17" s="8"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
+        <v>1073</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>1091</v>
+      </c>
+      <c r="C18" s="7">
+        <v>502</v>
+      </c>
+      <c r="D18" s="8"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D8"/>

</xml_diff>

<commit_message>
feat: update C-load HMI protocol, sync Excel map, add claude skills
- PlcProtocol.cs: C-load redesigned to DO 1pt (CMD) + DI 4pt (RESULT/MC1_FB/MC2_FB/SCR_FB) per stage
- Protection DI/DO addresses shifted +2 for PNL-1 (56-72), PNL-2/3 (24-40)
- RLC_IO_Protocol_Map.xlsx 05_ModbusBitMap synced to match HMI protocol
- MeteringView: trend chart max data point limit applied on double-click expand
- MainWindow: NaviFrame.Navigate → Content= for journal-free navigation
- CLAUDE.md: skill usage rule added (suggest registered skills on match)
- .claude/skills: new-skill, sync-protocol, design-worktree skills added

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Document/RLC_IO_Protocol_Map.xlsx
+++ b/Document/RLC_IO_Protocol_Map.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\1. RLC\RLC_LoadBank_SeparateVer\Document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A30C358-4D05-4BC1-A14B-9B3FBF8AC2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87C78681-099F-414F-AB40-8BD85CCFBBA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_분석요약" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6548" uniqueCount="1098">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6548" uniqueCount="1238">
   <si>
     <t>항목</t>
   </si>
@@ -3340,14 +3340,576 @@
     <t>PLC_03</t>
   </si>
   <si>
-    <t>192.168.1.1</t>
+    <t>P1_C1_RESULT</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>192.168.1.2</t>
-  </si>
-  <si>
-    <t>192.168.1.3</t>
+    <t>C부하 STEP1 동작 결과 (T=동작, F=멈춤)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_C1_MC1_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>C부하 STEP1 저항경유 MC 보조접점</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_C1_MC2_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>C부하 STEP1 직결 MC 보조접점</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_C2_RESULT</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>C부하 STEP2 동작 결과 (T=동작, F=멈춤)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_C2_MC1_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>C부하 STEP2 저항경유 MC 보조접점</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_C2_MC2_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>C부하 STEP2 직결 MC 보조접점</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_C1_SCR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>C부하 STEP1 SCR 게이팅 상태</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_C2_SCR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>C부하 STEP2 SCR 게이팅 상태</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_OVR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>과전압 계전기(OVR) 동작 접점</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_OCR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>과전류 계전기(OCR) 동작 접점</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_HT_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>과열(HT) 검출 접점</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_FAN_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>FAN 종합 운전 상태 피드백</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_MCCB_ON_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>MCCB ON 보조접점</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_MCCB_OFF_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>MCCB OFF 보조접점</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_MCCB_TRIP_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>MCCB TRIP 접점</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_EMG_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>비상정지(EMG STOP) 스위치 접점</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_DOOR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Door interlock 접점</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_FAN_R_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>R부하 냉각팬 운전 피드백</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_FAN_L_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>L부하 냉각팬 운전 피드백</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_FAN_C_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>C부하 냉각팬 운전 피드백</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_PWR_380_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>380V 주전원 투입 상태</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_PWR_220_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>220V 제어전원 투입 상태</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_CTRL_380_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>제어전원 380V(내부 변압기) 선택 상태</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_CTRL_220_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>제어전원 220V(외부전원) 선택 상태</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_LOC_REM_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>제어방식 선택 (0=Local, 1=Remote)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_C1_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>C부하 STEP1 투입/개방 명령</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>-</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Spare (예비)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>N</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_C2_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>C부하 STEP2 투입/개방 명령</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_FAN_R_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>R부하 냉각팬 기동 명령</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_FAN_L_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>L부하 냉각팬 기동 명령</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_FAN_C_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>C부하 냉각팬 기동 명령</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_MCCB_ON_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>MCCB ON 명령</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_MCCB_OFF_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>MCCB OFF 명령</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_MCCB_TRIP_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>MCCB TRIP 명령</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P1_RESET_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reset(고장 리셋) 명령</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_C1_RESULT</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_C1_MC1_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_C1_MC2_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_C2_RESULT</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_C2_MC1_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_C2_MC2_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_C1_SCR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_C2_SCR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_OVR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_OCR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_HT_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_FAN_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_MCCB_ON_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_MCCB_OFF_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_MCCB_TRIP_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_EMG_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_DOOR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_FAN_R_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_FAN_L_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_FAN_C_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_PWR_380_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_PWR_220_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_CTRL_380_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_CTRL_220_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_LOC_REM_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_C1_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_C2_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_FAN_R_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_FAN_L_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_FAN_C_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_MCCB_ON_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_MCCB_OFF_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_MCCB_TRIP_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P2_RESET_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_C1_RESULT</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_C1_MC1_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_C1_MC2_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_C2_RESULT</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_C2_MC1_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_C2_MC2_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_C1_SCR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_C2_SCR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_OVR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_OCR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_HT_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_FAN_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_MCCB_ON_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_MCCB_OFF_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_MCCB_TRIP_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_EMG_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_DOOR_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_FAN_R_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_FAN_L_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_FAN_C_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_PWR_380_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_PWR_220_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_CTRL_380_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_CTRL_220_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_LOC_REM_FB</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_C1_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_C2_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_FAN_R_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_FAN_L_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_FAN_C_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_MCCB_ON_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_MCCB_OFF_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_MCCB_TRIP_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>P3_RESET_CMD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>192.168.1.30</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>192.168.1.31</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>192.168.1.32</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -3355,9 +3917,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="178" formatCode="0_);[Red]\(0\)"/>
+    <numFmt numFmtId="176" formatCode="0_);[Red]\(0\)"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3382,6 +3944,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
@@ -3457,11 +4027,8 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3469,11 +4036,14 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4300,7 +4870,7 @@
     <col min="4" max="4" width="16.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1059</v>
       </c>
@@ -4317,46 +4887,46 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="9" t="s">
         <v>1092</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>1095</v>
-      </c>
-      <c r="C2" s="5">
+      <c r="B2" s="9" t="s">
+        <v>1235</v>
+      </c>
+      <c r="C2" s="9">
         <v>502</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="9" t="s">
         <v>1093</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>1096</v>
-      </c>
-      <c r="C3" s="5">
+      <c r="B3" s="9" t="s">
+        <v>1236</v>
+      </c>
+      <c r="C3" s="9">
         <v>502</v>
       </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="9" t="s">
         <v>1094</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>1097</v>
-      </c>
-      <c r="C4" s="5">
+      <c r="B4" s="9" t="s">
+        <v>1237</v>
+      </c>
+      <c r="C4" s="9">
         <v>502</v>
       </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
@@ -4503,62 +5073,62 @@
       <c r="F14" s="3"/>
     </row>
     <row r="15" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="6" t="s">
         <v>1070</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="6" t="s">
         <v>1088</v>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="6">
         <v>502</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="7" t="s">
         <v>1077</v>
       </c>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="6" t="s">
         <v>1071</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="6" t="s">
         <v>1089</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="6">
         <v>502</v>
       </c>
-      <c r="D16" s="8"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="6" t="s">
         <v>1072</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="6" t="s">
         <v>1090</v>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="6">
         <v>502</v>
       </c>
-      <c r="D17" s="8"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="6" t="s">
         <v>1073</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>1091</v>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="6">
         <v>502</v>
       </c>
-      <c r="D18" s="8"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
@@ -19365,16 +19935,16 @@
         <v>261</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>262</v>
+        <v>1095</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>263</v>
+        <v>1096</v>
       </c>
       <c r="I50" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
@@ -19397,16 +19967,16 @@
         <v>265</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>266</v>
+        <v>1098</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>267</v>
+        <v>1099</v>
       </c>
       <c r="I51" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
@@ -19429,16 +19999,16 @@
         <v>270</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>271</v>
+        <v>1100</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>272</v>
+        <v>1101</v>
       </c>
       <c r="I52" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
@@ -19461,16 +20031,16 @@
         <v>273</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>274</v>
+        <v>1102</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>275</v>
+        <v>1103</v>
       </c>
       <c r="I53" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.3">
@@ -19493,16 +20063,16 @@
         <v>276</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>277</v>
+        <v>1104</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>278</v>
+        <v>1105</v>
       </c>
       <c r="I54" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
@@ -19525,16 +20095,16 @@
         <v>280</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>281</v>
+        <v>1106</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>282</v>
+        <v>1107</v>
       </c>
       <c r="I55" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
@@ -19557,16 +20127,16 @@
         <v>283</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>284</v>
+        <v>1108</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>285</v>
+        <v>1109</v>
       </c>
       <c r="I56" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
@@ -19589,16 +20159,16 @@
         <v>288</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>289</v>
+        <v>1110</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>290</v>
+        <v>1111</v>
       </c>
       <c r="I57" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
@@ -19621,16 +20191,16 @@
         <v>291</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>292</v>
+        <v>1112</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>293</v>
+        <v>1113</v>
       </c>
       <c r="I58" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
@@ -19653,16 +20223,16 @@
         <v>295</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>296</v>
+        <v>1114</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>297</v>
+        <v>1115</v>
       </c>
       <c r="I59" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.3">
@@ -19685,16 +20255,16 @@
         <v>299</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>300</v>
+        <v>1116</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>301</v>
+        <v>1117</v>
       </c>
       <c r="I60" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.3">
@@ -19717,16 +20287,16 @@
         <v>304</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>305</v>
+        <v>1118</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>306</v>
+        <v>1119</v>
       </c>
       <c r="I61" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.3">
@@ -19749,16 +20319,16 @@
         <v>307</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>308</v>
+        <v>1120</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>309</v>
+        <v>1121</v>
       </c>
       <c r="I62" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.3">
@@ -19781,16 +20351,16 @@
         <v>311</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>312</v>
+        <v>1122</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>313</v>
+        <v>1123</v>
       </c>
       <c r="I63" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
@@ -19813,16 +20383,16 @@
         <v>315</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>316</v>
+        <v>1124</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>317</v>
+        <v>1125</v>
       </c>
       <c r="I64" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J64" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
@@ -19845,16 +20415,16 @@
         <v>318</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>319</v>
+        <v>1126</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>320</v>
+        <v>1127</v>
       </c>
       <c r="I65" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J65" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.3">
@@ -19877,16 +20447,16 @@
         <v>321</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>322</v>
+        <v>1128</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>323</v>
+        <v>1129</v>
       </c>
       <c r="I66" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J66" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
@@ -19909,16 +20479,16 @@
         <v>324</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>325</v>
+        <v>1130</v>
       </c>
       <c r="H67" s="2" t="s">
-        <v>326</v>
+        <v>1131</v>
       </c>
       <c r="I67" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J67" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
@@ -19941,16 +20511,16 @@
         <v>327</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>328</v>
+        <v>1132</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>329</v>
+        <v>1133</v>
       </c>
       <c r="I68" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J68" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
@@ -19973,16 +20543,16 @@
         <v>330</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>331</v>
+        <v>1134</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>332</v>
+        <v>1135</v>
       </c>
       <c r="I69" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J69" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
@@ -20005,16 +20575,16 @@
         <v>333</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>334</v>
+        <v>1136</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>335</v>
+        <v>1137</v>
       </c>
       <c r="I70" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J70" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
@@ -20037,16 +20607,16 @@
         <v>336</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>337</v>
+        <v>1138</v>
       </c>
       <c r="H71" s="2" t="s">
-        <v>338</v>
+        <v>1139</v>
       </c>
       <c r="I71" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J71" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
@@ -20069,16 +20639,16 @@
         <v>339</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>340</v>
+        <v>1140</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>341</v>
+        <v>1141</v>
       </c>
       <c r="I72" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J72" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
@@ -20101,16 +20671,16 @@
         <v>343</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>344</v>
+        <v>1142</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>345</v>
+        <v>1143</v>
       </c>
       <c r="I73" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J73" s="2" t="s">
-        <v>346</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
@@ -20133,16 +20703,16 @@
         <v>350</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>344</v>
+        <v>1144</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>345</v>
+        <v>1145</v>
       </c>
       <c r="I74" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J74" s="2" t="s">
-        <v>346</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.3">
@@ -21925,16 +22495,16 @@
         <v>505</v>
       </c>
       <c r="G130" s="2" t="s">
-        <v>506</v>
+        <v>1146</v>
       </c>
       <c r="H130" s="2" t="s">
-        <v>507</v>
+        <v>1147</v>
       </c>
       <c r="I130" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J130" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.3">
@@ -21957,16 +22527,16 @@
         <v>508</v>
       </c>
       <c r="G131" s="2" t="s">
-        <v>509</v>
+        <v>1148</v>
       </c>
       <c r="H131" s="2" t="s">
-        <v>510</v>
+        <v>1149</v>
       </c>
       <c r="I131" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J131" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.3">
@@ -21989,16 +22559,16 @@
         <v>511</v>
       </c>
       <c r="G132" s="2" t="s">
-        <v>512</v>
+        <v>1148</v>
       </c>
       <c r="H132" s="2" t="s">
-        <v>513</v>
+        <v>1149</v>
       </c>
       <c r="I132" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J132" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.3">
@@ -22021,16 +22591,16 @@
         <v>514</v>
       </c>
       <c r="G133" s="2" t="s">
-        <v>515</v>
+        <v>1151</v>
       </c>
       <c r="H133" s="2" t="s">
-        <v>516</v>
+        <v>1152</v>
       </c>
       <c r="I133" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J133" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.3">
@@ -22053,16 +22623,16 @@
         <v>517</v>
       </c>
       <c r="G134" s="2" t="s">
-        <v>518</v>
+        <v>1148</v>
       </c>
       <c r="H134" s="2" t="s">
-        <v>519</v>
+        <v>1149</v>
       </c>
       <c r="I134" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J134" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.3">
@@ -22085,16 +22655,16 @@
         <v>520</v>
       </c>
       <c r="G135" s="2" t="s">
-        <v>521</v>
+        <v>1148</v>
       </c>
       <c r="H135" s="2" t="s">
-        <v>522</v>
+        <v>1149</v>
       </c>
       <c r="I135" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J135" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.3">
@@ -22117,16 +22687,16 @@
         <v>523</v>
       </c>
       <c r="G136" s="2" t="s">
-        <v>524</v>
+        <v>1148</v>
       </c>
       <c r="H136" s="2" t="s">
-        <v>525</v>
+        <v>1149</v>
       </c>
       <c r="I136" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J136" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.3">
@@ -22149,16 +22719,16 @@
         <v>527</v>
       </c>
       <c r="G137" s="2" t="s">
-        <v>528</v>
+        <v>1148</v>
       </c>
       <c r="H137" s="2" t="s">
-        <v>529</v>
+        <v>1149</v>
       </c>
       <c r="I137" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J137" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.3">
@@ -22181,16 +22751,16 @@
         <v>530</v>
       </c>
       <c r="G138" s="2" t="s">
-        <v>531</v>
+        <v>1153</v>
       </c>
       <c r="H138" s="2" t="s">
-        <v>532</v>
+        <v>1154</v>
       </c>
       <c r="I138" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J138" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.3">
@@ -22213,16 +22783,16 @@
         <v>533</v>
       </c>
       <c r="G139" s="2" t="s">
-        <v>534</v>
+        <v>1155</v>
       </c>
       <c r="H139" s="2" t="s">
-        <v>535</v>
+        <v>1156</v>
       </c>
       <c r="I139" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J139" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.3">
@@ -22245,16 +22815,16 @@
         <v>536</v>
       </c>
       <c r="G140" s="2" t="s">
-        <v>537</v>
+        <v>1157</v>
       </c>
       <c r="H140" s="2" t="s">
-        <v>538</v>
+        <v>1158</v>
       </c>
       <c r="I140" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J140" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.3">
@@ -22277,16 +22847,16 @@
         <v>539</v>
       </c>
       <c r="G141" s="2" t="s">
-        <v>540</v>
+        <v>1159</v>
       </c>
       <c r="H141" s="2" t="s">
-        <v>541</v>
+        <v>1160</v>
       </c>
       <c r="I141" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J141" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.3">
@@ -22309,16 +22879,16 @@
         <v>542</v>
       </c>
       <c r="G142" s="2" t="s">
-        <v>543</v>
+        <v>1161</v>
       </c>
       <c r="H142" s="2" t="s">
-        <v>544</v>
+        <v>1162</v>
       </c>
       <c r="I142" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J142" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.3">
@@ -22341,16 +22911,16 @@
         <v>545</v>
       </c>
       <c r="G143" s="2" t="s">
-        <v>344</v>
+        <v>1163</v>
       </c>
       <c r="H143" s="2" t="s">
-        <v>345</v>
+        <v>1164</v>
       </c>
       <c r="I143" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J143" s="2" t="s">
-        <v>346</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="144" spans="1:10" x14ac:dyDescent="0.3">
@@ -22373,16 +22943,16 @@
         <v>546</v>
       </c>
       <c r="G144" s="2" t="s">
-        <v>344</v>
+        <v>1165</v>
       </c>
       <c r="H144" s="2" t="s">
-        <v>345</v>
+        <v>1166</v>
       </c>
       <c r="I144" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J144" s="2" t="s">
-        <v>346</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.3">
@@ -22949,16 +23519,16 @@
         <v>596</v>
       </c>
       <c r="G162" s="2" t="s">
-        <v>597</v>
+        <v>1167</v>
       </c>
       <c r="H162" s="2" t="s">
-        <v>263</v>
+        <v>1096</v>
       </c>
       <c r="I162" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J162" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="163" spans="1:10" x14ac:dyDescent="0.3">
@@ -22981,16 +23551,16 @@
         <v>598</v>
       </c>
       <c r="G163" s="2" t="s">
-        <v>599</v>
+        <v>1168</v>
       </c>
       <c r="H163" s="2" t="s">
-        <v>267</v>
+        <v>1099</v>
       </c>
       <c r="I163" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J163" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.3">
@@ -23013,16 +23583,16 @@
         <v>600</v>
       </c>
       <c r="G164" s="2" t="s">
-        <v>601</v>
+        <v>1169</v>
       </c>
       <c r="H164" s="2" t="s">
-        <v>272</v>
+        <v>1101</v>
       </c>
       <c r="I164" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J164" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="165" spans="1:10" x14ac:dyDescent="0.3">
@@ -23045,16 +23615,16 @@
         <v>602</v>
       </c>
       <c r="G165" s="2" t="s">
-        <v>603</v>
+        <v>1170</v>
       </c>
       <c r="H165" s="2" t="s">
-        <v>275</v>
+        <v>1103</v>
       </c>
       <c r="I165" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J165" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="166" spans="1:10" x14ac:dyDescent="0.3">
@@ -23077,16 +23647,16 @@
         <v>604</v>
       </c>
       <c r="G166" s="2" t="s">
-        <v>605</v>
+        <v>1171</v>
       </c>
       <c r="H166" s="2" t="s">
-        <v>278</v>
+        <v>1105</v>
       </c>
       <c r="I166" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J166" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="167" spans="1:10" x14ac:dyDescent="0.3">
@@ -23109,16 +23679,16 @@
         <v>606</v>
       </c>
       <c r="G167" s="2" t="s">
-        <v>607</v>
+        <v>1172</v>
       </c>
       <c r="H167" s="2" t="s">
-        <v>282</v>
+        <v>1107</v>
       </c>
       <c r="I167" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J167" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="168" spans="1:10" x14ac:dyDescent="0.3">
@@ -23141,16 +23711,16 @@
         <v>608</v>
       </c>
       <c r="G168" s="2" t="s">
-        <v>609</v>
+        <v>1173</v>
       </c>
       <c r="H168" s="2" t="s">
-        <v>285</v>
+        <v>1109</v>
       </c>
       <c r="I168" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J168" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="169" spans="1:10" x14ac:dyDescent="0.3">
@@ -23173,16 +23743,16 @@
         <v>610</v>
       </c>
       <c r="G169" s="2" t="s">
-        <v>611</v>
+        <v>1174</v>
       </c>
       <c r="H169" s="2" t="s">
-        <v>290</v>
+        <v>1111</v>
       </c>
       <c r="I169" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J169" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.3">
@@ -23205,16 +23775,16 @@
         <v>612</v>
       </c>
       <c r="G170" s="2" t="s">
-        <v>613</v>
+        <v>1175</v>
       </c>
       <c r="H170" s="2" t="s">
-        <v>293</v>
+        <v>1113</v>
       </c>
       <c r="I170" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J170" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="171" spans="1:10" x14ac:dyDescent="0.3">
@@ -23237,16 +23807,16 @@
         <v>614</v>
       </c>
       <c r="G171" s="2" t="s">
-        <v>615</v>
+        <v>1176</v>
       </c>
       <c r="H171" s="2" t="s">
-        <v>297</v>
+        <v>1115</v>
       </c>
       <c r="I171" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J171" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="172" spans="1:10" x14ac:dyDescent="0.3">
@@ -23269,16 +23839,16 @@
         <v>616</v>
       </c>
       <c r="G172" s="2" t="s">
-        <v>617</v>
+        <v>1177</v>
       </c>
       <c r="H172" s="2" t="s">
-        <v>301</v>
+        <v>1117</v>
       </c>
       <c r="I172" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J172" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="173" spans="1:10" x14ac:dyDescent="0.3">
@@ -23301,16 +23871,16 @@
         <v>618</v>
       </c>
       <c r="G173" s="2" t="s">
-        <v>619</v>
+        <v>1178</v>
       </c>
       <c r="H173" s="2" t="s">
-        <v>306</v>
+        <v>1119</v>
       </c>
       <c r="I173" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J173" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="174" spans="1:10" x14ac:dyDescent="0.3">
@@ -23333,16 +23903,16 @@
         <v>620</v>
       </c>
       <c r="G174" s="2" t="s">
-        <v>621</v>
+        <v>1179</v>
       </c>
       <c r="H174" s="2" t="s">
-        <v>309</v>
+        <v>1121</v>
       </c>
       <c r="I174" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J174" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="175" spans="1:10" x14ac:dyDescent="0.3">
@@ -23365,16 +23935,16 @@
         <v>622</v>
       </c>
       <c r="G175" s="2" t="s">
-        <v>623</v>
+        <v>1180</v>
       </c>
       <c r="H175" s="2" t="s">
-        <v>313</v>
+        <v>1123</v>
       </c>
       <c r="I175" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J175" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="176" spans="1:10" x14ac:dyDescent="0.3">
@@ -23397,16 +23967,16 @@
         <v>624</v>
       </c>
       <c r="G176" s="2" t="s">
-        <v>625</v>
+        <v>1181</v>
       </c>
       <c r="H176" s="2" t="s">
-        <v>317</v>
+        <v>1125</v>
       </c>
       <c r="I176" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J176" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="177" spans="1:10" x14ac:dyDescent="0.3">
@@ -23429,16 +23999,16 @@
         <v>626</v>
       </c>
       <c r="G177" s="2" t="s">
-        <v>627</v>
+        <v>1182</v>
       </c>
       <c r="H177" s="2" t="s">
-        <v>320</v>
+        <v>1127</v>
       </c>
       <c r="I177" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J177" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="178" spans="1:10" x14ac:dyDescent="0.3">
@@ -23461,16 +24031,16 @@
         <v>628</v>
       </c>
       <c r="G178" s="2" t="s">
-        <v>629</v>
+        <v>1183</v>
       </c>
       <c r="H178" s="2" t="s">
-        <v>323</v>
+        <v>1129</v>
       </c>
       <c r="I178" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J178" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="179" spans="1:10" x14ac:dyDescent="0.3">
@@ -23493,16 +24063,16 @@
         <v>630</v>
       </c>
       <c r="G179" s="2" t="s">
-        <v>631</v>
+        <v>1184</v>
       </c>
       <c r="H179" s="2" t="s">
-        <v>326</v>
+        <v>1131</v>
       </c>
       <c r="I179" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J179" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="180" spans="1:10" x14ac:dyDescent="0.3">
@@ -23525,16 +24095,16 @@
         <v>632</v>
       </c>
       <c r="G180" s="2" t="s">
-        <v>633</v>
+        <v>1185</v>
       </c>
       <c r="H180" s="2" t="s">
-        <v>329</v>
+        <v>1133</v>
       </c>
       <c r="I180" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J180" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="181" spans="1:10" x14ac:dyDescent="0.3">
@@ -23557,16 +24127,16 @@
         <v>634</v>
       </c>
       <c r="G181" s="2" t="s">
-        <v>635</v>
+        <v>1186</v>
       </c>
       <c r="H181" s="2" t="s">
-        <v>332</v>
+        <v>1135</v>
       </c>
       <c r="I181" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J181" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="182" spans="1:10" x14ac:dyDescent="0.3">
@@ -23589,16 +24159,16 @@
         <v>636</v>
       </c>
       <c r="G182" s="2" t="s">
-        <v>637</v>
+        <v>1187</v>
       </c>
       <c r="H182" s="2" t="s">
-        <v>335</v>
+        <v>1137</v>
       </c>
       <c r="I182" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J182" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="183" spans="1:10" x14ac:dyDescent="0.3">
@@ -23621,16 +24191,16 @@
         <v>638</v>
       </c>
       <c r="G183" s="2" t="s">
-        <v>639</v>
+        <v>1188</v>
       </c>
       <c r="H183" s="2" t="s">
-        <v>338</v>
+        <v>1139</v>
       </c>
       <c r="I183" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J183" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="184" spans="1:10" x14ac:dyDescent="0.3">
@@ -23653,16 +24223,16 @@
         <v>640</v>
       </c>
       <c r="G184" s="2" t="s">
-        <v>641</v>
+        <v>1189</v>
       </c>
       <c r="H184" s="2" t="s">
-        <v>341</v>
+        <v>1141</v>
       </c>
       <c r="I184" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J184" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="185" spans="1:10" x14ac:dyDescent="0.3">
@@ -23685,16 +24255,16 @@
         <v>642</v>
       </c>
       <c r="G185" s="2" t="s">
-        <v>344</v>
+        <v>1190</v>
       </c>
       <c r="H185" s="2" t="s">
-        <v>345</v>
+        <v>1143</v>
       </c>
       <c r="I185" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J185" s="2" t="s">
-        <v>346</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="186" spans="1:10" x14ac:dyDescent="0.3">
@@ -23717,16 +24287,16 @@
         <v>643</v>
       </c>
       <c r="G186" s="2" t="s">
-        <v>344</v>
+        <v>1191</v>
       </c>
       <c r="H186" s="2" t="s">
-        <v>345</v>
+        <v>1145</v>
       </c>
       <c r="I186" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J186" s="2" t="s">
-        <v>346</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="187" spans="1:10" x14ac:dyDescent="0.3">
@@ -24485,16 +25055,16 @@
         <v>699</v>
       </c>
       <c r="G210" s="2" t="s">
-        <v>700</v>
+        <v>1192</v>
       </c>
       <c r="H210" s="2" t="s">
-        <v>507</v>
+        <v>1147</v>
       </c>
       <c r="I210" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J210" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="211" spans="1:10" x14ac:dyDescent="0.3">
@@ -24517,16 +25087,16 @@
         <v>701</v>
       </c>
       <c r="G211" s="2" t="s">
-        <v>702</v>
+        <v>1193</v>
       </c>
       <c r="H211" s="2" t="s">
-        <v>510</v>
+        <v>1152</v>
       </c>
       <c r="I211" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J211" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="212" spans="1:10" x14ac:dyDescent="0.3">
@@ -24549,16 +25119,16 @@
         <v>703</v>
       </c>
       <c r="G212" s="2" t="s">
-        <v>704</v>
+        <v>1148</v>
       </c>
       <c r="H212" s="2" t="s">
-        <v>513</v>
+        <v>1149</v>
       </c>
       <c r="I212" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J212" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="213" spans="1:10" x14ac:dyDescent="0.3">
@@ -24581,16 +25151,16 @@
         <v>705</v>
       </c>
       <c r="G213" s="2" t="s">
-        <v>706</v>
+        <v>1148</v>
       </c>
       <c r="H213" s="2" t="s">
-        <v>516</v>
+        <v>1149</v>
       </c>
       <c r="I213" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J213" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="214" spans="1:10" x14ac:dyDescent="0.3">
@@ -24613,16 +25183,16 @@
         <v>707</v>
       </c>
       <c r="G214" s="2" t="s">
-        <v>708</v>
+        <v>1148</v>
       </c>
       <c r="H214" s="2" t="s">
-        <v>519</v>
+        <v>1149</v>
       </c>
       <c r="I214" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J214" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="215" spans="1:10" x14ac:dyDescent="0.3">
@@ -24645,16 +25215,16 @@
         <v>709</v>
       </c>
       <c r="G215" s="2" t="s">
-        <v>710</v>
+        <v>1148</v>
       </c>
       <c r="H215" s="2" t="s">
-        <v>522</v>
+        <v>1149</v>
       </c>
       <c r="I215" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J215" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="216" spans="1:10" x14ac:dyDescent="0.3">
@@ -24677,16 +25247,16 @@
         <v>711</v>
       </c>
       <c r="G216" s="2" t="s">
-        <v>712</v>
+        <v>1148</v>
       </c>
       <c r="H216" s="2" t="s">
-        <v>525</v>
+        <v>1149</v>
       </c>
       <c r="I216" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J216" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="217" spans="1:10" x14ac:dyDescent="0.3">
@@ -24709,16 +25279,16 @@
         <v>713</v>
       </c>
       <c r="G217" s="2" t="s">
-        <v>714</v>
+        <v>1148</v>
       </c>
       <c r="H217" s="2" t="s">
-        <v>529</v>
+        <v>1149</v>
       </c>
       <c r="I217" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J217" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="218" spans="1:10" x14ac:dyDescent="0.3">
@@ -24741,16 +25311,16 @@
         <v>715</v>
       </c>
       <c r="G218" s="2" t="s">
-        <v>716</v>
+        <v>1194</v>
       </c>
       <c r="H218" s="2" t="s">
-        <v>532</v>
+        <v>1154</v>
       </c>
       <c r="I218" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J218" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="219" spans="1:10" x14ac:dyDescent="0.3">
@@ -24773,16 +25343,16 @@
         <v>717</v>
       </c>
       <c r="G219" s="2" t="s">
-        <v>718</v>
+        <v>1195</v>
       </c>
       <c r="H219" s="2" t="s">
-        <v>535</v>
+        <v>1156</v>
       </c>
       <c r="I219" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J219" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="220" spans="1:10" x14ac:dyDescent="0.3">
@@ -24805,16 +25375,16 @@
         <v>719</v>
       </c>
       <c r="G220" s="2" t="s">
-        <v>720</v>
+        <v>1196</v>
       </c>
       <c r="H220" s="2" t="s">
-        <v>538</v>
+        <v>1158</v>
       </c>
       <c r="I220" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J220" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="221" spans="1:10" x14ac:dyDescent="0.3">
@@ -24837,16 +25407,16 @@
         <v>721</v>
       </c>
       <c r="G221" s="2" t="s">
-        <v>722</v>
+        <v>1197</v>
       </c>
       <c r="H221" s="2" t="s">
-        <v>541</v>
+        <v>1160</v>
       </c>
       <c r="I221" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J221" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="222" spans="1:10" x14ac:dyDescent="0.3">
@@ -24869,16 +25439,16 @@
         <v>723</v>
       </c>
       <c r="G222" s="2" t="s">
-        <v>724</v>
+        <v>1198</v>
       </c>
       <c r="H222" s="2" t="s">
-        <v>544</v>
+        <v>1162</v>
       </c>
       <c r="I222" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J222" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="223" spans="1:10" x14ac:dyDescent="0.3">
@@ -24901,16 +25471,16 @@
         <v>725</v>
       </c>
       <c r="G223" s="2" t="s">
-        <v>344</v>
+        <v>1199</v>
       </c>
       <c r="H223" s="2" t="s">
-        <v>345</v>
+        <v>1164</v>
       </c>
       <c r="I223" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J223" s="2" t="s">
-        <v>346</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="224" spans="1:10" x14ac:dyDescent="0.3">
@@ -24933,16 +25503,16 @@
         <v>726</v>
       </c>
       <c r="G224" s="2" t="s">
-        <v>344</v>
+        <v>1200</v>
       </c>
       <c r="H224" s="2" t="s">
-        <v>345</v>
+        <v>1166</v>
       </c>
       <c r="I224" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J224" s="2" t="s">
-        <v>346</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="225" spans="1:10" x14ac:dyDescent="0.3">
@@ -25509,16 +26079,16 @@
         <v>760</v>
       </c>
       <c r="G242" s="2" t="s">
-        <v>761</v>
+        <v>1201</v>
       </c>
       <c r="H242" s="2" t="s">
-        <v>263</v>
+        <v>1096</v>
       </c>
       <c r="I242" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J242" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="243" spans="1:10" x14ac:dyDescent="0.3">
@@ -25541,16 +26111,16 @@
         <v>762</v>
       </c>
       <c r="G243" s="2" t="s">
-        <v>763</v>
+        <v>1202</v>
       </c>
       <c r="H243" s="2" t="s">
-        <v>267</v>
+        <v>1099</v>
       </c>
       <c r="I243" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J243" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="244" spans="1:10" x14ac:dyDescent="0.3">
@@ -25573,16 +26143,16 @@
         <v>764</v>
       </c>
       <c r="G244" s="2" t="s">
-        <v>765</v>
+        <v>1203</v>
       </c>
       <c r="H244" s="2" t="s">
-        <v>272</v>
+        <v>1101</v>
       </c>
       <c r="I244" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J244" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="245" spans="1:10" x14ac:dyDescent="0.3">
@@ -25605,16 +26175,16 @@
         <v>766</v>
       </c>
       <c r="G245" s="2" t="s">
-        <v>767</v>
+        <v>1204</v>
       </c>
       <c r="H245" s="2" t="s">
-        <v>275</v>
+        <v>1103</v>
       </c>
       <c r="I245" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J245" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="246" spans="1:10" x14ac:dyDescent="0.3">
@@ -25637,16 +26207,16 @@
         <v>768</v>
       </c>
       <c r="G246" s="2" t="s">
-        <v>769</v>
+        <v>1205</v>
       </c>
       <c r="H246" s="2" t="s">
-        <v>278</v>
+        <v>1105</v>
       </c>
       <c r="I246" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J246" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="247" spans="1:10" x14ac:dyDescent="0.3">
@@ -25669,16 +26239,16 @@
         <v>770</v>
       </c>
       <c r="G247" s="2" t="s">
-        <v>771</v>
+        <v>1206</v>
       </c>
       <c r="H247" s="2" t="s">
-        <v>282</v>
+        <v>1107</v>
       </c>
       <c r="I247" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J247" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="248" spans="1:10" x14ac:dyDescent="0.3">
@@ -25701,16 +26271,16 @@
         <v>772</v>
       </c>
       <c r="G248" s="2" t="s">
-        <v>773</v>
+        <v>1207</v>
       </c>
       <c r="H248" s="2" t="s">
-        <v>285</v>
+        <v>1109</v>
       </c>
       <c r="I248" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J248" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="249" spans="1:10" x14ac:dyDescent="0.3">
@@ -25733,16 +26303,16 @@
         <v>774</v>
       </c>
       <c r="G249" s="2" t="s">
-        <v>775</v>
+        <v>1208</v>
       </c>
       <c r="H249" s="2" t="s">
-        <v>290</v>
+        <v>1111</v>
       </c>
       <c r="I249" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J249" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="250" spans="1:10" x14ac:dyDescent="0.3">
@@ -25765,16 +26335,16 @@
         <v>776</v>
       </c>
       <c r="G250" s="2" t="s">
-        <v>777</v>
+        <v>1209</v>
       </c>
       <c r="H250" s="2" t="s">
-        <v>293</v>
+        <v>1113</v>
       </c>
       <c r="I250" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J250" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="251" spans="1:10" x14ac:dyDescent="0.3">
@@ -25797,16 +26367,16 @@
         <v>778</v>
       </c>
       <c r="G251" s="2" t="s">
-        <v>779</v>
+        <v>1210</v>
       </c>
       <c r="H251" s="2" t="s">
-        <v>297</v>
+        <v>1115</v>
       </c>
       <c r="I251" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J251" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="252" spans="1:10" x14ac:dyDescent="0.3">
@@ -25829,16 +26399,16 @@
         <v>780</v>
       </c>
       <c r="G252" s="2" t="s">
-        <v>781</v>
+        <v>1211</v>
       </c>
       <c r="H252" s="2" t="s">
-        <v>301</v>
+        <v>1117</v>
       </c>
       <c r="I252" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J252" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="253" spans="1:10" x14ac:dyDescent="0.3">
@@ -25861,16 +26431,16 @@
         <v>782</v>
       </c>
       <c r="G253" s="2" t="s">
-        <v>783</v>
+        <v>1212</v>
       </c>
       <c r="H253" s="2" t="s">
-        <v>306</v>
+        <v>1119</v>
       </c>
       <c r="I253" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J253" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="254" spans="1:10" x14ac:dyDescent="0.3">
@@ -25893,16 +26463,16 @@
         <v>784</v>
       </c>
       <c r="G254" s="2" t="s">
-        <v>785</v>
+        <v>1213</v>
       </c>
       <c r="H254" s="2" t="s">
-        <v>309</v>
+        <v>1121</v>
       </c>
       <c r="I254" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J254" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="255" spans="1:10" x14ac:dyDescent="0.3">
@@ -25925,16 +26495,16 @@
         <v>786</v>
       </c>
       <c r="G255" s="2" t="s">
-        <v>787</v>
+        <v>1214</v>
       </c>
       <c r="H255" s="2" t="s">
-        <v>313</v>
+        <v>1123</v>
       </c>
       <c r="I255" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J255" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="256" spans="1:10" x14ac:dyDescent="0.3">
@@ -25957,16 +26527,16 @@
         <v>788</v>
       </c>
       <c r="G256" s="2" t="s">
-        <v>789</v>
+        <v>1215</v>
       </c>
       <c r="H256" s="2" t="s">
-        <v>317</v>
+        <v>1125</v>
       </c>
       <c r="I256" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J256" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="257" spans="1:10" x14ac:dyDescent="0.3">
@@ -25989,16 +26559,16 @@
         <v>790</v>
       </c>
       <c r="G257" s="2" t="s">
-        <v>791</v>
+        <v>1216</v>
       </c>
       <c r="H257" s="2" t="s">
-        <v>320</v>
+        <v>1127</v>
       </c>
       <c r="I257" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J257" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="258" spans="1:10" x14ac:dyDescent="0.3">
@@ -26021,16 +26591,16 @@
         <v>792</v>
       </c>
       <c r="G258" s="2" t="s">
-        <v>793</v>
+        <v>1217</v>
       </c>
       <c r="H258" s="2" t="s">
-        <v>323</v>
+        <v>1129</v>
       </c>
       <c r="I258" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J258" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="259" spans="1:10" x14ac:dyDescent="0.3">
@@ -26053,16 +26623,16 @@
         <v>794</v>
       </c>
       <c r="G259" s="2" t="s">
-        <v>795</v>
+        <v>1218</v>
       </c>
       <c r="H259" s="2" t="s">
-        <v>326</v>
+        <v>1131</v>
       </c>
       <c r="I259" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J259" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="260" spans="1:10" x14ac:dyDescent="0.3">
@@ -26085,16 +26655,16 @@
         <v>796</v>
       </c>
       <c r="G260" s="2" t="s">
-        <v>797</v>
+        <v>1219</v>
       </c>
       <c r="H260" s="2" t="s">
-        <v>329</v>
+        <v>1133</v>
       </c>
       <c r="I260" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J260" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="261" spans="1:10" x14ac:dyDescent="0.3">
@@ -26117,16 +26687,16 @@
         <v>798</v>
       </c>
       <c r="G261" s="2" t="s">
-        <v>799</v>
+        <v>1220</v>
       </c>
       <c r="H261" s="2" t="s">
-        <v>332</v>
+        <v>1135</v>
       </c>
       <c r="I261" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J261" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="262" spans="1:10" x14ac:dyDescent="0.3">
@@ -26149,16 +26719,16 @@
         <v>800</v>
       </c>
       <c r="G262" s="2" t="s">
-        <v>801</v>
+        <v>1221</v>
       </c>
       <c r="H262" s="2" t="s">
-        <v>335</v>
+        <v>1137</v>
       </c>
       <c r="I262" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J262" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="263" spans="1:10" x14ac:dyDescent="0.3">
@@ -26181,16 +26751,16 @@
         <v>802</v>
       </c>
       <c r="G263" s="2" t="s">
-        <v>803</v>
+        <v>1222</v>
       </c>
       <c r="H263" s="2" t="s">
-        <v>338</v>
+        <v>1139</v>
       </c>
       <c r="I263" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J263" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="264" spans="1:10" x14ac:dyDescent="0.3">
@@ -26213,16 +26783,16 @@
         <v>804</v>
       </c>
       <c r="G264" s="2" t="s">
-        <v>805</v>
+        <v>1223</v>
       </c>
       <c r="H264" s="2" t="s">
-        <v>341</v>
+        <v>1141</v>
       </c>
       <c r="I264" s="2" t="s">
         <v>880</v>
       </c>
       <c r="J264" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="265" spans="1:10" x14ac:dyDescent="0.3">
@@ -26245,16 +26815,16 @@
         <v>806</v>
       </c>
       <c r="G265" s="2" t="s">
-        <v>344</v>
+        <v>1224</v>
       </c>
       <c r="H265" s="2" t="s">
-        <v>345</v>
+        <v>1143</v>
       </c>
       <c r="I265" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J265" s="2" t="s">
-        <v>346</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="266" spans="1:10" x14ac:dyDescent="0.3">
@@ -26277,16 +26847,16 @@
         <v>807</v>
       </c>
       <c r="G266" s="2" t="s">
-        <v>344</v>
+        <v>1225</v>
       </c>
       <c r="H266" s="2" t="s">
-        <v>345</v>
+        <v>1145</v>
       </c>
       <c r="I266" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J266" s="2" t="s">
-        <v>346</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="267" spans="1:10" x14ac:dyDescent="0.3">
@@ -27045,16 +27615,16 @@
         <v>847</v>
       </c>
       <c r="G290" s="2" t="s">
-        <v>848</v>
+        <v>1226</v>
       </c>
       <c r="H290" s="2" t="s">
-        <v>507</v>
+        <v>1147</v>
       </c>
       <c r="I290" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J290" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="291" spans="1:10" x14ac:dyDescent="0.3">
@@ -27077,16 +27647,16 @@
         <v>849</v>
       </c>
       <c r="G291" s="2" t="s">
-        <v>850</v>
+        <v>1227</v>
       </c>
       <c r="H291" s="2" t="s">
-        <v>510</v>
+        <v>1152</v>
       </c>
       <c r="I291" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J291" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="292" spans="1:10" x14ac:dyDescent="0.3">
@@ -27109,16 +27679,16 @@
         <v>851</v>
       </c>
       <c r="G292" s="2" t="s">
-        <v>852</v>
+        <v>1148</v>
       </c>
       <c r="H292" s="2" t="s">
-        <v>513</v>
+        <v>1149</v>
       </c>
       <c r="I292" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J292" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="293" spans="1:10" x14ac:dyDescent="0.3">
@@ -27141,16 +27711,16 @@
         <v>853</v>
       </c>
       <c r="G293" s="2" t="s">
-        <v>854</v>
+        <v>1148</v>
       </c>
       <c r="H293" s="2" t="s">
-        <v>516</v>
+        <v>1149</v>
       </c>
       <c r="I293" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J293" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="294" spans="1:10" x14ac:dyDescent="0.3">
@@ -27173,16 +27743,16 @@
         <v>855</v>
       </c>
       <c r="G294" s="2" t="s">
-        <v>856</v>
+        <v>1148</v>
       </c>
       <c r="H294" s="2" t="s">
-        <v>519</v>
+        <v>1149</v>
       </c>
       <c r="I294" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J294" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="295" spans="1:10" x14ac:dyDescent="0.3">
@@ -27205,16 +27775,16 @@
         <v>857</v>
       </c>
       <c r="G295" s="2" t="s">
-        <v>858</v>
+        <v>1148</v>
       </c>
       <c r="H295" s="2" t="s">
-        <v>522</v>
+        <v>1149</v>
       </c>
       <c r="I295" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J295" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="296" spans="1:10" x14ac:dyDescent="0.3">
@@ -27237,16 +27807,16 @@
         <v>859</v>
       </c>
       <c r="G296" s="2" t="s">
-        <v>860</v>
+        <v>1148</v>
       </c>
       <c r="H296" s="2" t="s">
-        <v>525</v>
+        <v>1149</v>
       </c>
       <c r="I296" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J296" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="297" spans="1:10" x14ac:dyDescent="0.3">
@@ -27269,16 +27839,16 @@
         <v>861</v>
       </c>
       <c r="G297" s="2" t="s">
-        <v>862</v>
+        <v>1148</v>
       </c>
       <c r="H297" s="2" t="s">
-        <v>529</v>
+        <v>1149</v>
       </c>
       <c r="I297" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J297" s="2" t="s">
-        <v>115</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="298" spans="1:10" x14ac:dyDescent="0.3">
@@ -27301,16 +27871,16 @@
         <v>863</v>
       </c>
       <c r="G298" s="2" t="s">
-        <v>864</v>
+        <v>1228</v>
       </c>
       <c r="H298" s="2" t="s">
-        <v>532</v>
+        <v>1154</v>
       </c>
       <c r="I298" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J298" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="299" spans="1:10" x14ac:dyDescent="0.3">
@@ -27333,16 +27903,16 @@
         <v>865</v>
       </c>
       <c r="G299" s="2" t="s">
-        <v>866</v>
+        <v>1229</v>
       </c>
       <c r="H299" s="2" t="s">
-        <v>535</v>
+        <v>1156</v>
       </c>
       <c r="I299" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J299" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="300" spans="1:10" x14ac:dyDescent="0.3">
@@ -27365,16 +27935,16 @@
         <v>867</v>
       </c>
       <c r="G300" s="2" t="s">
-        <v>868</v>
+        <v>1230</v>
       </c>
       <c r="H300" s="2" t="s">
-        <v>538</v>
+        <v>1158</v>
       </c>
       <c r="I300" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J300" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="301" spans="1:10" x14ac:dyDescent="0.3">
@@ -27397,16 +27967,16 @@
         <v>869</v>
       </c>
       <c r="G301" s="2" t="s">
-        <v>870</v>
+        <v>1231</v>
       </c>
       <c r="H301" s="2" t="s">
-        <v>541</v>
+        <v>1160</v>
       </c>
       <c r="I301" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J301" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="302" spans="1:10" x14ac:dyDescent="0.3">
@@ -27429,16 +27999,16 @@
         <v>871</v>
       </c>
       <c r="G302" s="2" t="s">
-        <v>872</v>
+        <v>1232</v>
       </c>
       <c r="H302" s="2" t="s">
-        <v>544</v>
+        <v>1162</v>
       </c>
       <c r="I302" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J302" s="2" t="s">
-        <v>115</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="303" spans="1:10" x14ac:dyDescent="0.3">
@@ -27461,16 +28031,16 @@
         <v>873</v>
       </c>
       <c r="G303" s="2" t="s">
-        <v>344</v>
+        <v>1233</v>
       </c>
       <c r="H303" s="2" t="s">
-        <v>345</v>
+        <v>1164</v>
       </c>
       <c r="I303" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J303" s="2" t="s">
-        <v>346</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="304" spans="1:10" x14ac:dyDescent="0.3">
@@ -27493,16 +28063,16 @@
         <v>874</v>
       </c>
       <c r="G304" s="2" t="s">
-        <v>344</v>
+        <v>1234</v>
       </c>
       <c r="H304" s="2" t="s">
-        <v>345</v>
+        <v>1166</v>
       </c>
       <c r="I304" s="2" t="s">
         <v>881</v>
       </c>
       <c r="J304" s="2" t="s">
-        <v>346</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="305" spans="1:10" x14ac:dyDescent="0.3">
@@ -27546,6 +28116,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:I120"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -29351,7 +29922,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>61</v>
       </c>
@@ -29380,7 +29951,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>61</v>
       </c>
@@ -29409,7 +29980,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>61</v>
       </c>
@@ -29438,7 +30009,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>61</v>
       </c>
@@ -29467,7 +30038,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>61</v>
       </c>
@@ -29496,7 +30067,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>61</v>
       </c>
@@ -29525,7 +30096,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>61</v>
       </c>
@@ -29554,7 +30125,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>61</v>
       </c>
@@ -29583,7 +30154,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>61</v>
       </c>
@@ -29612,7 +30183,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>61</v>
       </c>
@@ -29641,7 +30212,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>61</v>
       </c>
@@ -29670,7 +30241,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>61</v>
       </c>
@@ -29699,7 +30270,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>61</v>
       </c>
@@ -29728,7 +30299,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>61</v>
       </c>
@@ -29757,7 +30328,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>61</v>
       </c>
@@ -29786,7 +30357,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>61</v>
       </c>
@@ -29815,7 +30386,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>61</v>
       </c>
@@ -29844,7 +30415,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>61</v>
       </c>
@@ -29873,7 +30444,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>61</v>
       </c>
@@ -29902,7 +30473,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>61</v>
       </c>
@@ -29931,7 +30502,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>61</v>
       </c>
@@ -29960,7 +30531,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>61</v>
       </c>
@@ -29989,7 +30560,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>61</v>
       </c>
@@ -30018,7 +30589,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>61</v>
       </c>
@@ -30047,7 +30618,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>61</v>
       </c>
@@ -30076,7 +30647,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>61</v>
       </c>
@@ -30105,7 +30676,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>61</v>
       </c>
@@ -30134,7 +30705,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>61</v>
       </c>
@@ -30163,7 +30734,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>61</v>
       </c>
@@ -30186,7 +30757,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>65</v>
       </c>
@@ -30215,7 +30786,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>65</v>
       </c>
@@ -30244,7 +30815,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
         <v>65</v>
       </c>
@@ -30273,7 +30844,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>65</v>
       </c>
@@ -30302,7 +30873,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>65</v>
       </c>
@@ -30331,7 +30902,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>65</v>
       </c>
@@ -30360,7 +30931,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>65</v>
       </c>
@@ -30389,7 +30960,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
         <v>65</v>
       </c>
@@ -30418,7 +30989,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>65</v>
       </c>
@@ -30447,7 +31018,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>65</v>
       </c>
@@ -30476,7 +31047,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>65</v>
       </c>
@@ -30505,7 +31076,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>65</v>
       </c>
@@ -30534,7 +31105,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
         <v>65</v>
       </c>
@@ -30563,7 +31134,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
         <v>65</v>
       </c>
@@ -30592,7 +31163,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
         <v>65</v>
       </c>
@@ -30621,7 +31192,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>65</v>
       </c>
@@ -30650,7 +31221,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
         <v>65</v>
       </c>
@@ -30679,7 +31250,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
         <v>65</v>
       </c>
@@ -30708,7 +31279,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
         <v>65</v>
       </c>
@@ -30737,7 +31308,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
         <v>65</v>
       </c>
@@ -30766,7 +31337,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>65</v>
       </c>
@@ -30795,7 +31366,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
         <v>65</v>
       </c>
@@ -30824,7 +31395,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
         <v>65</v>
       </c>
@@ -30853,7 +31424,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
         <v>65</v>
       </c>
@@ -30882,7 +31453,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
         <v>65</v>
       </c>
@@ -30911,7 +31482,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
         <v>65</v>
       </c>
@@ -30940,7 +31511,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
         <v>65</v>
       </c>
@@ -30969,7 +31540,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
         <v>65</v>
       </c>
@@ -30998,7 +31569,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
         <v>65</v>
       </c>
@@ -31022,7 +31593,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I120" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <autoFilter ref="A1:I120" xr:uid="{00000000-0009-0000-0000-000006000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="PNL-1"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>